<commit_message>
Update cost planner to compare deployment options
Update the cost planner spreadsheet to include a comparison between Autoscale and Reserved VM deployment types for estimating platform costs.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: c963a842-7f06-460a-8dd2-f4e7a2c98973
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c786953a-a967-479d-a1c8-d26552ded4ee
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/121eda0a-d7e2-4425-ab2e-aa06a7816154/c963a842-7f06-460a-8dd2-f4e7a2c98973/LNkmzzf
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Shepherd_Connect_Annual_Cost_Planner.xlsx
+++ b/Shepherd_Connect_Annual_Cost_Planner.xlsx
@@ -13,6 +13,7 @@
     <sheet name="📲 Termii Calculator" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="📅 Monthly Schedule" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="🇳🇬 NGN Conversion" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="⚖️ Deployment Comparison" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="168" formatCode="&quot;₦&quot;#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,20 @@
       <color rgb="006B7280"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00EA580C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -176,6 +189,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
         <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000EA5E9"/>
+        <bgColor rgb="000EA5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0016A34A"/>
+        <bgColor rgb="0016A34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
   </fills>
@@ -263,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -467,6 +498,96 @@
     </xf>
     <xf numFmtId="168" fontId="11" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1019,10 +1140,7 @@
     </row>
     <row r="6" ht="22" customHeight="1"/>
     <row r="7" ht="22" customHeight="1"/>
-    <row r="8">
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
@@ -1078,10 +1196,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
@@ -1607,7 +1722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F24"/>
+  <dimension ref="B1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1890,6 +2005,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="4" customHeight="1"/>
     <row r="21" ht="24" customHeight="1">
       <c r="B21" s="32" t="inlineStr">
@@ -1924,6 +2040,7 @@
       </c>
       <c r="E22" s="38" t="inlineStr"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="B24" s="16" t="inlineStr">
         <is>
@@ -1934,6 +2051,51 @@
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="13" t="n"/>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B17:E17"/>
@@ -2867,6 +3029,12 @@
           <t>⭐  First-year cost also includes one-time upfront Termii pre-load buffer (see '💰 Cost Summary' sheet · '⭐ FIRST-YEAR TOTAL' row).</t>
         </is>
       </c>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="16" t="inlineStr">
@@ -2874,6 +3042,12 @@
           <t>💡  PAYG top-up tip: When your Termii balance drops below the monthly buffer amount, top up immediately. Set a Termii low-balance alert in the dashboard to get notified before you run out. Recommended minimum top-up: $50 at a time.</t>
         </is>
       </c>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3059,4 +3233,634 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000891B2"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="B1" s="76" t="inlineStr">
+        <is>
+          <t>⚖️  AUTOSCALE (PAYG)  vs  RESERVED VM — Which is right for you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="B2" s="77" t="inlineStr">
+        <is>
+          <t>Both options require Replit Core ($18/month). Yellow cells are editable estimates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="78" t="inlineStr">
+        <is>
+          <t>⚡ AUTOSCALE (PAYG)</t>
+        </is>
+      </c>
+      <c r="F4" s="79" t="inlineStr">
+        <is>
+          <t>🖥️ RESERVED VM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="80" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C5" s="80" t="inlineStr">
+        <is>
+          <t>Monthly (USD)</t>
+        </is>
+      </c>
+      <c r="D5" s="80" t="inlineStr">
+        <is>
+          <t>Annual (USD)</t>
+        </is>
+      </c>
+      <c r="F5" s="81" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="G5" s="81" t="inlineStr">
+        <is>
+          <t>Monthly (USD)</t>
+        </is>
+      </c>
+      <c r="H5" s="81" t="inlineStr">
+        <is>
+          <t>Annual (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>Replit Core subscription</t>
+        </is>
+      </c>
+      <c r="C6" s="83">
+        <f>'💰 Cost Summary'!C4</f>
+        <v/>
+      </c>
+      <c r="D6" s="83">
+        <f>'💰 Cost Summary'!D4</f>
+        <v/>
+      </c>
+      <c r="F6" s="84" t="inlineStr">
+        <is>
+          <t>Replit Core subscription</t>
+        </is>
+      </c>
+      <c r="G6" s="85">
+        <f>'💰 Cost Summary'!C4</f>
+        <v/>
+      </c>
+      <c r="H6" s="85">
+        <f>'💰 Cost Summary'!D4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="86" t="inlineStr">
+        <is>
+          <t>Sunday compute — est. cost per Sunday</t>
+        </is>
+      </c>
+      <c r="C7" s="87" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="88">
+        <f>C7*12</f>
+        <v/>
+      </c>
+      <c r="F7" s="86" t="inlineStr">
+        <is>
+          <t>Reserved VM — 1 vCPU / 1 GB  ✅ recommended</t>
+        </is>
+      </c>
+      <c r="G7" s="87" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" s="88">
+        <f>G7*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × avg Sundays per month</t>
+        </is>
+      </c>
+      <c r="C8" s="89" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D8" s="83">
+        <f>C8*12</f>
+        <v/>
+      </c>
+      <c r="F8" s="84" t="inlineStr">
+        <is>
+          <t>Reserved VM — 2 vCPU / 2 GB  (comfortable headroom)</t>
+        </is>
+      </c>
+      <c r="G8" s="87" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" s="85">
+        <f>G8*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sunday compute subtotal</t>
+        </is>
+      </c>
+      <c r="C9" s="88">
+        <f>C7*C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="88">
+        <f>C7*C8*12</f>
+        <v/>
+      </c>
+      <c r="F9" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Use ONE of the two tiers above in your budget</t>
+        </is>
+      </c>
+      <c r="G9" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="88" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="82" t="inlineStr">
+        <is>
+          <t>Weekday low-traffic compute (est.)</t>
+        </is>
+      </c>
+      <c r="C10" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="83">
+        <f>C10*12</f>
+        <v/>
+      </c>
+      <c r="F10" s="84" t="inlineStr">
+        <is>
+          <t>Termii (SMS + Email + WA + Buffer)</t>
+        </is>
+      </c>
+      <c r="G10" s="85">
+        <f>('💰 Cost Summary'!C6+'💰 Cost Summary'!C9+'💰 Cost Summary'!C12+'💰 Cost Summary'!C15)</f>
+        <v/>
+      </c>
+      <c r="H10" s="85">
+        <f>('💰 Cost Summary'!D6+'💰 Cost Summary'!D9+'💰 Cost Summary'!D12+'💰 Cost Summary'!D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="86" t="inlineStr">
+        <is>
+          <t>Termii (SMS + Email + WA + Buffer)</t>
+        </is>
+      </c>
+      <c r="C11" s="88">
+        <f>('💰 Cost Summary'!C6+'💰 Cost Summary'!C9+'💰 Cost Summary'!C12+'💰 Cost Summary'!C15)</f>
+        <v/>
+      </c>
+      <c r="D11" s="88">
+        <f>('💰 Cost Summary'!D6+'💰 Cost Summary'!D9+'💰 Cost Summary'!D12+'💰 Cost Summary'!D15)</f>
+        <v/>
+      </c>
+      <c r="F11" s="86" t="inlineStr">
+        <is>
+          <t>Custom domain (optional)</t>
+        </is>
+      </c>
+      <c r="G11" s="88">
+        <f>ROUND('⚙️ Assumptions'!C28/12,2)</f>
+        <v/>
+      </c>
+      <c r="H11" s="88">
+        <f>'⚙️ Assumptions'!C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="B12" s="82" t="inlineStr">
+        <is>
+          <t>Custom domain (optional)</t>
+        </is>
+      </c>
+      <c r="C12" s="83">
+        <f>ROUND('⚙️ Assumptions'!C28/12,2)</f>
+        <v/>
+      </c>
+      <c r="D12" s="83">
+        <f>'⚙️ Assumptions'!C28</f>
+        <v/>
+      </c>
+      <c r="F12" s="91" t="inlineStr">
+        <is>
+          <t>🖥️  RESERVED VM TOTAL (1 vCPU)</t>
+        </is>
+      </c>
+      <c r="G12" s="92">
+        <f>SUM(G6,G7,G10,G11)</f>
+        <v/>
+      </c>
+      <c r="H12" s="92">
+        <f>SUM(H6,H7,H10,H11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="93" t="inlineStr">
+        <is>
+          <t>⚡  AUTOSCALE TOTAL</t>
+        </is>
+      </c>
+      <c r="C13" s="94">
+        <f>SUM(C6,C9,C10,C11,C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="94">
+        <f>SUM(D6,D9,D10,D11,D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="95" t="inlineStr">
+        <is>
+          <t>📊  FEATURE &amp; COST COMPARISON</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="96" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C15" s="97" t="inlineStr">
+        <is>
+          <t>⚡ Autoscale</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="98" t="inlineStr">
+        <is>
+          <t>🖥️ Reserved VM</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="99" t="inlineStr">
+        <is>
+          <t>Billing model</t>
+        </is>
+      </c>
+      <c r="C16" s="100" t="inlineStr">
+        <is>
+          <t>Pay per compute second</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="100" t="inlineStr">
+        <is>
+          <t>Fixed monthly fee</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="13" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="101" t="inlineStr">
+        <is>
+          <t>Estimated monthly platform</t>
+        </is>
+      </c>
+      <c r="C17" s="102">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="102">
+        <f>G12</f>
+        <v/>
+      </c>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="13" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="99" t="inlineStr">
+        <is>
+          <t>Estimated annual platform</t>
+        </is>
+      </c>
+      <c r="C18" s="103">
+        <f>D13</f>
+        <v/>
+      </c>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="103">
+        <f>H12</f>
+        <v/>
+      </c>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="13" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="101" t="inlineStr">
+        <is>
+          <t>Possible annual saving</t>
+        </is>
+      </c>
+      <c r="C19" s="102">
+        <f>H12-D13 (if +ve, Autoscale wins)</f>
+        <v/>
+      </c>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="104" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="99" t="inlineStr">
+        <is>
+          <t>Traffic handling</t>
+        </is>
+      </c>
+      <c r="C20" s="100" t="inlineStr">
+        <is>
+          <t>Auto-scales to any demand ✅</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="100" t="inlineStr">
+        <is>
+          <t>Fixed capacity — sized at setup</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="13" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="101" t="inlineStr">
+        <is>
+          <t>Handles Sunday peak?</t>
+        </is>
+      </c>
+      <c r="C21" s="104" t="inlineStr">
+        <is>
+          <t>Yes — scales instantly ✅</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="104" t="inlineStr">
+        <is>
+          <t>Yes — 1 vCPU handles ~500 concurrent ✅</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="13" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="99" t="inlineStr">
+        <is>
+          <t>Idle time billing</t>
+        </is>
+      </c>
+      <c r="C22" s="100" t="inlineStr">
+        <is>
+          <t>Near-zero on quiet weekdays ✅</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="100" t="inlineStr">
+        <is>
+          <t>Full price 24/7 even when idle</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="13" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="101" t="inlineStr">
+        <is>
+          <t>Budget predictability</t>
+        </is>
+      </c>
+      <c r="C23" s="104" t="inlineStr">
+        <is>
+          <t>Varies (~$23–35/mo est.)</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="104" t="inlineStr">
+        <is>
+          <t>100% fixed — zero surprises ✅</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="99" t="inlineStr">
+        <is>
+          <t>Best for</t>
+        </is>
+      </c>
+      <c r="C24" s="100" t="inlineStr">
+        <is>
+          <t>Low-traffic-except-Sundays pattern ✅</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="100" t="inlineStr">
+        <is>
+          <t>Church finance team prefers fixed bills ✅</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="13" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="101" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="C25" s="104" t="inlineStr">
+        <is>
+          <t>Surprise bill if unusual event</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="104" t="inlineStr">
+        <is>
+          <t>Over-paying on quiet months</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="13" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="99" t="inlineStr">
+        <is>
+          <t>Database included?</t>
+        </is>
+      </c>
+      <c r="C26" s="100" t="inlineStr">
+        <is>
+          <t>Yes (Core plan) ✅</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="100" t="inlineStr">
+        <is>
+          <t>Yes (Core plan) ✅</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="13" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="101" t="inlineStr">
+        <is>
+          <t>Object storage included?</t>
+        </is>
+      </c>
+      <c r="C27" s="104" t="inlineStr">
+        <is>
+          <t>Yes — 50 GB (Core plan) ✅</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="104" t="inlineStr">
+        <is>
+          <t>Yes — 50 GB (Core plan) ✅</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="13" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="99" t="inlineStr">
+        <is>
+          <t>Recommended for 2,000 users?</t>
+        </is>
+      </c>
+      <c r="C28" s="100" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="100" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="13" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="105" t="inlineStr">
+        <is>
+          <t>⚠️  Yellow cells are editable. Change Sunday compute cost and VM tier to match your actual Replit bill. Termii figures are pulled live from your Assumptions sheet. Replit publishes current deployment pricing at replit.com/pricing.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="34">
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="F24:H24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>